<commit_message>
new field added for filter and issue fixed
</commit_message>
<xml_diff>
--- a/Presentation/Visitor.API/FormatFiles/Template_Visitor.xlsx
+++ b/Presentation/Visitor.API/FormatFiles/Template_Visitor.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="90">
   <si>
     <t>VisitorName</t>
   </si>
@@ -274,6 +274,18 @@
   </si>
   <si>
     <t>28/12/2025</t>
+  </si>
+  <si>
+    <t>28/08/2025 10:05:10 AM</t>
+  </si>
+  <si>
+    <t>28/08/2025 06:15:50 PM</t>
+  </si>
+  <si>
+    <t>28/08/2025 08:25:40 PM</t>
+  </si>
+  <si>
+    <t>28/08/2025 09:15:20 AM</t>
   </si>
 </sst>
 </file>
@@ -682,8 +694,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
@@ -835,10 +847,10 @@
         <v>59</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>60</v>
@@ -945,10 +957,10 @@
         <v>61</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>62</v>

</xml_diff>